<commit_message>
docs: update panel dataset with new CPU data (Gavriilidis et al 2026, through 2026)
</commit_message>
<xml_diff>
--- a/uploads/east_asia_panel_fixed.xlsx
+++ b/uploads/east_asia_panel_fixed.xlsx
@@ -531,7 +531,7 @@
         <v>20.414</v>
       </c>
       <c r="D2" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E2" t="n">
         <v>0.2565059792250396</v>
@@ -595,7 +595,7 @@
         <v>18.414</v>
       </c>
       <c r="D3" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E3" t="n">
         <v>0.2652939409017562</v>
@@ -659,7 +659,7 @@
         <v>17.367</v>
       </c>
       <c r="D4" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E4" t="n">
         <v>0.2205440501372018</v>
@@ -723,7 +723,7 @@
         <v>18.751</v>
       </c>
       <c r="D5" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E5" t="n">
         <v>0.2434430072704952</v>
@@ -787,7 +787,7 @@
         <v>18.137</v>
       </c>
       <c r="D6" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E6" t="n">
         <v>0.2662028148770332</v>
@@ -851,7 +851,7 @@
         <v>19.286</v>
       </c>
       <c r="D7" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E7" t="n">
         <v>0.190336737781763</v>
@@ -915,7 +915,7 @@
         <v>17.535</v>
       </c>
       <c r="D8" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E8" t="n">
         <v>0.2561134124795595</v>
@@ -979,7 +979,7 @@
         <v>17.517</v>
       </c>
       <c r="D9" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E9" t="n">
         <v>0.2077676796664793</v>
@@ -1043,7 +1043,7 @@
         <v>17.287</v>
       </c>
       <c r="D10" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E10" t="n">
         <v>0.3124568065007527</v>
@@ -1107,7 +1107,7 @@
         <v>16.105</v>
       </c>
       <c r="D11" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E11" t="n">
         <v>0.3886795764168104</v>
@@ -1171,7 +1171,7 @@
         <v>16.639</v>
       </c>
       <c r="D12" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E12" t="n">
         <v>0.2434541657567022</v>
@@ -1235,7 +1235,7 @@
         <v>18.958</v>
       </c>
       <c r="D13" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E13" t="n">
         <v>0.3796609255174796</v>
@@ -1299,7 +1299,7 @@
         <v>17.618</v>
       </c>
       <c r="D14" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E14" t="n">
         <v>0.3378655426204203</v>
@@ -1363,7 +1363,7 @@
         <v>15.036</v>
       </c>
       <c r="D15" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E15" t="n">
         <v>0.5473370353380841</v>
@@ -1427,7 +1427,7 @@
         <v>16.222</v>
       </c>
       <c r="D16" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E16" t="n">
         <v>0.3740352143843967</v>
@@ -1491,7 +1491,7 @@
         <v>16.173</v>
       </c>
       <c r="D17" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E17" t="n">
         <v>0.4370223904649418</v>
@@ -1555,7 +1555,7 @@
         <v>15.588</v>
       </c>
       <c r="D18" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E18" t="n">
         <v>0.5760255853335065</v>
@@ -1619,7 +1619,7 @@
         <v>15.258</v>
       </c>
       <c r="D19" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E19" t="n">
         <v>0.4216572592655818</v>
@@ -1683,7 +1683,7 @@
         <v>19.025</v>
       </c>
       <c r="D20" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E20" t="n">
         <v>0.3497177809476852</v>
@@ -1747,7 +1747,7 @@
         <v>17.886</v>
       </c>
       <c r="D21" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E21" t="n">
         <v>0.3957575969398021</v>
@@ -1811,7 +1811,7 @@
         <v>18.691</v>
       </c>
       <c r="D22" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E22" t="n">
         <v>0.4341458032528559</v>
@@ -1875,7 +1875,7 @@
         <v>16.813</v>
       </c>
       <c r="D23" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E23" t="n">
         <v>0.3831185537079968</v>
@@ -1939,7 +1939,7 @@
         <v>20.041</v>
       </c>
       <c r="D24" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E24" t="n">
         <v>0.4896654635667801</v>
@@ -2003,7 +2003,7 @@
         <v>20.13</v>
       </c>
       <c r="D25" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E25" t="n">
         <v>0.3884186769525208</v>
@@ -2067,7 +2067,7 @@
         <v>22.249</v>
       </c>
       <c r="D26" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E26" t="n">
         <v>0.3794428904851279</v>
@@ -2131,7 +2131,7 @@
         <v>23.968</v>
       </c>
       <c r="D27" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E27" t="n">
         <v>0.4124086573719979</v>
@@ -2195,7 +2195,7 @@
         <v>24.829</v>
       </c>
       <c r="D28" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E28" t="n">
         <v>0.449655329187711</v>
@@ -2259,7 +2259,7 @@
         <v>25.242</v>
       </c>
       <c r="D29" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E29" t="n">
         <v>0.8143434425195055</v>
@@ -2323,7 +2323,7 @@
         <v>25.612</v>
       </c>
       <c r="D30" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E30" t="n">
         <v>0.9167053649822868</v>
@@ -2387,7 +2387,7 @@
         <v>26.85</v>
       </c>
       <c r="D31" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E31" t="n">
         <v>0.8645223677158366</v>
@@ -2451,7 +2451,7 @@
         <v>28.088</v>
       </c>
       <c r="D32" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E32" t="n">
         <v>0.7542644441127774</v>
@@ -2515,7 +2515,7 @@
         <v>28.694</v>
       </c>
       <c r="D33" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E33" t="n">
         <v>0.7334313392639161</v>
@@ -2579,7 +2579,7 @@
         <v>30.181</v>
       </c>
       <c r="D34" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E34" t="n">
         <v>1.176426768302918</v>
@@ -2643,7 +2643,7 @@
         <v>30.606</v>
       </c>
       <c r="D35" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E35" t="n">
         <v>1.053532282511394</v>
@@ -2707,7 +2707,7 @@
         <v>33.696</v>
       </c>
       <c r="D36" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E36" t="n">
         <v>0.8718154033025104</v>
@@ -2771,7 +2771,7 @@
         <v>23.01</v>
       </c>
       <c r="D37" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E37" t="n">
         <v>0.0338453355555733</v>
@@ -2835,7 +2835,7 @@
         <v>22.205</v>
       </c>
       <c r="D38" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E38" t="n">
         <v>0.0311058829538524</v>
@@ -2899,7 +2899,7 @@
         <v>26.639</v>
       </c>
       <c r="D39" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E39" t="n">
         <v>0.0217193634792541</v>
@@ -2963,7 +2963,7 @@
         <v>25.142</v>
       </c>
       <c r="D40" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E40" t="n">
         <v>0.0226891544492294</v>
@@ -3027,7 +3027,7 @@
         <v>20.873</v>
       </c>
       <c r="D41" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E41" t="n">
         <v>0.0319963354462136</v>
@@ -3091,7 +3091,7 @@
         <v>19.412</v>
       </c>
       <c r="D42" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E42" t="n">
         <v>0.027836095696936</v>
@@ -3155,7 +3155,7 @@
         <v>18.97</v>
       </c>
       <c r="D43" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E43" t="n">
         <v>0.0393578958852837</v>
@@ -3219,7 +3219,7 @@
         <v>12.157</v>
       </c>
       <c r="D44" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E44" t="n">
         <v>0.0358111890964209</v>
@@ -3283,7 +3283,7 @@
         <v>17.798</v>
       </c>
       <c r="D45" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E45" t="n">
         <v>0.0666575717429319</v>
@@ -3347,7 +3347,7 @@
         <v>17.054</v>
       </c>
       <c r="D46" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E46" t="n">
         <v>0.09870410834749541</v>
@@ -3411,7 +3411,7 @@
         <v>19.992</v>
       </c>
       <c r="D47" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E47" t="n">
         <v>0.0492260662528376</v>
@@ -3475,7 +3475,7 @@
         <v>20.902</v>
       </c>
       <c r="D48" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E48" t="n">
         <v>0.0883251704896489</v>
@@ -3539,7 +3539,7 @@
         <v>18.577</v>
       </c>
       <c r="D49" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E49" t="n">
         <v>0.123823834117502</v>
@@ -3603,7 +3603,7 @@
         <v>16.884</v>
       </c>
       <c r="D50" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E50" t="n">
         <v>0.1225423840805887</v>
@@ -3667,7 +3667,7 @@
         <v>16.806</v>
       </c>
       <c r="D51" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E51" t="n">
         <v>0.0920447555060189</v>
@@ -3731,7 +3731,7 @@
         <v>17.052</v>
       </c>
       <c r="D52" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E52" t="n">
         <v>0.0867505713055531</v>
@@ -3795,7 +3795,7 @@
         <v>15.348</v>
       </c>
       <c r="D53" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E53" t="n">
         <v>0.06395321773986019</v>
@@ -3859,7 +3859,7 @@
         <v>16.368</v>
       </c>
       <c r="D54" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E54" t="n">
         <v>0.0439268518239259</v>
@@ -3923,7 +3923,7 @@
         <v>16.895</v>
       </c>
       <c r="D55" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E55" t="n">
         <v>0.0414783246815204</v>
@@ -3987,7 +3987,7 @@
         <v>16.449</v>
       </c>
       <c r="D56" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E56" t="n">
         <v>0.0459643892633418</v>
@@ -4051,7 +4051,7 @@
         <v>19.503</v>
       </c>
       <c r="D57" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E57" t="n">
         <v>0.0331261022171626</v>
@@ -4115,7 +4115,7 @@
         <v>15.875</v>
       </c>
       <c r="D58" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E58" t="n">
         <v>0.034250598711272</v>
@@ -4179,7 +4179,7 @@
         <v>14.888</v>
       </c>
       <c r="D59" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E59" t="n">
         <v>0.0213128506826857</v>
@@ -4243,7 +4243,7 @@
         <v>15.765</v>
       </c>
       <c r="D60" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E60" t="n">
         <v>0.0158325436059385</v>
@@ -4307,7 +4307,7 @@
         <v>14.486</v>
       </c>
       <c r="D61" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E61" t="n">
         <v>0.0316599870566278</v>
@@ -4371,7 +4371,7 @@
         <v>13.795</v>
       </c>
       <c r="D62" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E62" t="n">
         <v>0.0193674179414908</v>
@@ -4435,7 +4435,7 @@
         <v>15.368</v>
       </c>
       <c r="D63" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E63" t="n">
         <v>0.0375975945498794</v>
@@ -4499,7 +4499,7 @@
         <v>16.247</v>
       </c>
       <c r="D64" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E64" t="n">
         <v>0.0361923112068325</v>
@@ -4563,7 +4563,7 @@
         <v>17.048</v>
       </c>
       <c r="D65" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E65" t="n">
         <v>0.0319729273129875</v>
@@ -4627,7 +4627,7 @@
         <v>16.26</v>
       </c>
       <c r="D66" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E66" t="n">
         <v>0.0361500372334072</v>
@@ -4691,7 +4691,7 @@
         <v>18.124</v>
       </c>
       <c r="D67" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E67" t="n">
         <v>0.023627788061276</v>
@@ -4755,7 +4755,7 @@
         <v>18.167</v>
       </c>
       <c r="D68" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E68" t="n">
         <v>0.023597480651612</v>
@@ -4819,7 +4819,7 @@
         <v>19.611</v>
       </c>
       <c r="D69" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E69" t="n">
         <v>0.09348709353556239</v>
@@ -4883,7 +4883,7 @@
         <v>18.597</v>
       </c>
       <c r="D70" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E70" t="n">
         <v>0.08016299052784839</v>
@@ -4947,7 +4947,7 @@
         <v>18.09</v>
       </c>
       <c r="D71" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E71" t="n">
         <v>0.0541130780863265</v>
@@ -5011,7 +5011,7 @@
         <v>11.144</v>
       </c>
       <c r="D72" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E72" t="n">
         <v>0.3953243506451446</v>
@@ -5075,7 +5075,7 @@
         <v>11.639</v>
       </c>
       <c r="D73" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E73" t="n">
         <v>0.3832643578449885</v>
@@ -5139,7 +5139,7 @@
         <v>10.025</v>
       </c>
       <c r="D74" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E74" t="n">
         <v>0.1940890364348887</v>
@@ -5203,7 +5203,7 @@
         <v>11.247</v>
       </c>
       <c r="D75" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E75" t="n">
         <v>0.2490083488325278</v>
@@ -5267,7 +5267,7 @@
         <v>7.919</v>
       </c>
       <c r="D76" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E76" t="n">
         <v>0.2606769303480786</v>
@@ -5331,7 +5331,7 @@
         <v>9.212999999999999</v>
       </c>
       <c r="D77" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E77" t="n">
         <v>0.2117192087074121</v>
@@ -5395,7 +5395,7 @@
         <v>8.98</v>
       </c>
       <c r="D78" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E78" t="n">
         <v>0.1604590406641363</v>
@@ -5459,7 +5459,7 @@
         <v>9.762</v>
       </c>
       <c r="D79" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E79" t="n">
         <v>0.1523053795099259</v>
@@ -5523,7 +5523,7 @@
         <v>9.946999999999999</v>
       </c>
       <c r="D80" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E80" t="n">
         <v>0.1580951778839032</v>
@@ -5587,7 +5587,7 @@
         <v>9.316000000000001</v>
       </c>
       <c r="D81" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E81" t="n">
         <v>0.151504099369049</v>
@@ -5651,7 +5651,7 @@
         <v>9.186999999999999</v>
       </c>
       <c r="D82" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E82" t="n">
         <v>0.1052139848470687</v>
@@ -5715,7 +5715,7 @@
         <v>9.077</v>
       </c>
       <c r="D83" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E83" t="n">
         <v>0.3306996825461584</v>
@@ -5779,7 +5779,7 @@
         <v>8.942</v>
       </c>
       <c r="D84" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E84" t="n">
         <v>0.3300629903872806</v>
@@ -5843,7 +5843,7 @@
         <v>10.263</v>
       </c>
       <c r="D85" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E85" t="n">
         <v>0.4845499793688457</v>
@@ -5907,7 +5907,7 @@
         <v>10.028</v>
       </c>
       <c r="D86" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E86" t="n">
         <v>0.2754493094980718</v>
@@ -5971,7 +5971,7 @@
         <v>8.914</v>
       </c>
       <c r="D87" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E87" t="n">
         <v>0.2298227474093437</v>
@@ -6035,7 +6035,7 @@
         <v>9.831</v>
       </c>
       <c r="D88" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E88" t="n">
         <v>0.26437298891445</v>
@@ -6099,7 +6099,7 @@
         <v>8.622999999999999</v>
       </c>
       <c r="D89" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E89" t="n">
         <v>0.1676841353376706</v>
@@ -6163,7 +6163,7 @@
         <v>8.615</v>
       </c>
       <c r="D90" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E90" t="n">
         <v>0.1383473258465529</v>
@@ -6227,7 +6227,7 @@
         <v>8.731999999999999</v>
       </c>
       <c r="D91" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E91" t="n">
         <v>0.1939563030997911</v>
@@ -6291,7 +6291,7 @@
         <v>10.228</v>
       </c>
       <c r="D92" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E92" t="n">
         <v>0.1617873571813106</v>
@@ -6355,7 +6355,7 @@
         <v>10.279</v>
       </c>
       <c r="D93" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E93" t="n">
         <v>0.1589114218950271</v>
@@ -6419,7 +6419,7 @@
         <v>10.058</v>
       </c>
       <c r="D94" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E94" t="n">
         <v>0.147398080676794</v>
@@ -6483,7 +6483,7 @@
         <v>11.082</v>
       </c>
       <c r="D95" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E95" t="n">
         <v>0.1730755778650442</v>
@@ -6547,7 +6547,7 @@
         <v>12.6</v>
       </c>
       <c r="D96" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E96" t="n">
         <v>0.1484907840689024</v>
@@ -6611,7 +6611,7 @@
         <v>14.952</v>
       </c>
       <c r="D97" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E97" t="n">
         <v>0.1432324089109898</v>
@@ -6675,7 +6675,7 @@
         <v>14.268</v>
       </c>
       <c r="D98" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E98" t="n">
         <v>0.2159111027916271</v>
@@ -6739,7 +6739,7 @@
         <v>15.164</v>
       </c>
       <c r="D99" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E99" t="n">
         <v>0.4278514459729194</v>
@@ -6803,7 +6803,7 @@
         <v>16.191</v>
       </c>
       <c r="D100" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E100" t="n">
         <v>0.3243980358044305</v>
@@ -6867,7 +6867,7 @@
         <v>16.843</v>
       </c>
       <c r="D101" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E101" t="n">
         <v>0.293594155460596</v>
@@ -6931,7 +6931,7 @@
         <v>19.092</v>
       </c>
       <c r="D102" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E102" t="n">
         <v>0.177309460317095</v>
@@ -6995,7 +6995,7 @@
         <v>20.117</v>
       </c>
       <c r="D103" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E103" t="n">
         <v>0.2176062961419424</v>
@@ -7059,7 +7059,7 @@
         <v>20.488</v>
       </c>
       <c r="D104" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E104" t="n">
         <v>0.3832631893455984</v>
@@ -7123,7 +7123,7 @@
         <v>22.137</v>
       </c>
       <c r="D105" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E105" t="n">
         <v>0.2764560406406721</v>
@@ -7187,7 +7187,7 @@
         <v>22.935</v>
       </c>
       <c r="D106" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E106" t="n">
         <v>0.1956517032037179</v>
@@ -7251,7 +7251,7 @@
         <v>3.955</v>
       </c>
       <c r="D107" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E107" t="n">
         <v>0.1398523083577553</v>
@@ -7315,7 +7315,7 @@
         <v>2.649</v>
       </c>
       <c r="D108" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E108" t="n">
         <v>0.1849058680236339</v>
@@ -7379,7 +7379,7 @@
         <v>2.117</v>
       </c>
       <c r="D109" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E109" t="n">
         <v>0.1273506979147592</v>
@@ -7443,7 +7443,7 @@
         <v>2.613</v>
       </c>
       <c r="D110" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E110" t="n">
         <v>0.2363762228439252</v>
@@ -7507,7 +7507,7 @@
         <v>1.281</v>
       </c>
       <c r="D111" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E111" t="n">
         <v>0.4049725383520122</v>
@@ -7571,7 +7571,7 @@
         <v>1.48</v>
       </c>
       <c r="D112" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E112" t="n">
         <v>0.1280991046999891</v>
@@ -7635,7 +7635,7 @@
         <v>1.253</v>
       </c>
       <c r="D113" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E113" t="n">
         <v>0.1058600200340151</v>
@@ -7699,7 +7699,7 @@
         <v>1.174</v>
       </c>
       <c r="D114" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E114" t="n">
         <v>0.09472967063387221</v>
@@ -7763,7 +7763,7 @@
         <v>1.831</v>
       </c>
       <c r="D115" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E115" t="n">
         <v>0.1229226669917503</v>
@@ -7827,7 +7827,7 @@
         <v>1.624</v>
       </c>
       <c r="D116" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E116" t="n">
         <v>0.1683059521019458</v>
@@ -7891,7 +7891,7 @@
         <v>1.418</v>
       </c>
       <c r="D117" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E117" t="n">
         <v>0.1462997831404208</v>
@@ -7955,7 +7955,7 @@
         <v>0.787</v>
       </c>
       <c r="D118" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E118" t="n">
         <v>0.197716308136781</v>
@@ -8019,7 +8019,7 @@
         <v>1.033</v>
       </c>
       <c r="D119" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E119" t="n">
         <v>0.3346020442744098</v>
@@ -8083,7 +8083,7 @@
         <v>1.469</v>
       </c>
       <c r="D120" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E120" t="n">
         <v>0.624695412814617</v>
@@ -8147,7 +8147,7 @@
         <v>1.266</v>
       </c>
       <c r="D121" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E121" t="n">
         <v>0.3262688716252643</v>
@@ -8211,7 +8211,7 @@
         <v>1.045</v>
       </c>
       <c r="D122" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E122" t="n">
         <v>0.2782472483813763</v>
@@ -8275,7 +8275,7 @@
         <v>0.988</v>
       </c>
       <c r="D123" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E123" t="n">
         <v>0.3845680033167204</v>
@@ -8339,7 +8339,7 @@
         <v>1.048</v>
       </c>
       <c r="D124" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E124" t="n">
         <v>0.2485717547436556</v>
@@ -8403,7 +8403,7 @@
         <v>1.003</v>
       </c>
       <c r="D125" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E125" t="n">
         <v>0.1758416158457596</v>
@@ -8467,7 +8467,7 @@
         <v>1.019</v>
       </c>
       <c r="D126" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E126" t="n">
         <v>0.3131593180199464</v>
@@ -8531,7 +8531,7 @@
         <v>1.149</v>
       </c>
       <c r="D127" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E127" t="n">
         <v>0.2765436898916961</v>
@@ -8595,7 +8595,7 @@
         <v>1.428</v>
       </c>
       <c r="D128" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E128" t="n">
         <v>0.1432179020096858</v>
@@ -8659,7 +8659,7 @@
         <v>1.538</v>
       </c>
       <c r="D129" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E129" t="n">
         <v>0.1618198913832505</v>
@@ -8723,7 +8723,7 @@
         <v>1.904</v>
       </c>
       <c r="D130" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E130" t="n">
         <v>0.2624897677451372</v>
@@ -8787,7 +8787,7 @@
         <v>2.385</v>
       </c>
       <c r="D131" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E131" t="n">
         <v>0.1274289687474568</v>
@@ -8851,7 +8851,7 @@
         <v>2.775</v>
       </c>
       <c r="D132" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E132" t="n">
         <v>0.1230600674947103</v>
@@ -8915,7 +8915,7 @@
         <v>3.232</v>
       </c>
       <c r="D133" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E133" t="n">
         <v>0.288712120304505</v>
@@ -8979,7 +8979,7 @@
         <v>3.874</v>
       </c>
       <c r="D134" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E134" t="n">
         <v>0.878054926792781</v>
@@ -9043,7 +9043,7 @@
         <v>4.689</v>
       </c>
       <c r="D135" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E135" t="n">
         <v>0.6790721168120699</v>
@@ -9107,7 +9107,7 @@
         <v>5.625</v>
       </c>
       <c r="D136" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E136" t="n">
         <v>0.3959129477540652</v>
@@ -9171,7 +9171,7 @@
         <v>7</v>
       </c>
       <c r="D137" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E137" t="n">
         <v>0.2115590088069439</v>
@@ -9235,7 +9235,7 @@
         <v>7.914</v>
       </c>
       <c r="D138" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E138" t="n">
         <v>0.2185384891927241</v>
@@ -9299,7 +9299,7 @@
         <v>8.913</v>
       </c>
       <c r="D139" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E139" t="n">
         <v>0.3623031166692576</v>
@@ -9363,7 +9363,7 @@
         <v>9.566000000000001</v>
       </c>
       <c r="D140" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E140" t="n">
         <v>0.3148706046243509</v>
@@ -9427,7 +9427,7 @@
         <v>9.709</v>
       </c>
       <c r="D141" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E141" t="n">
         <v>0.3382945768535136</v>
@@ -9491,7 +9491,7 @@
         <v>17.495</v>
       </c>
       <c r="D142" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E142" t="n">
         <v>0.0239790513878688</v>
@@ -9555,7 +9555,7 @@
         <v>16.757</v>
       </c>
       <c r="D143" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E143" t="n">
         <v>0.0196326779356847</v>
@@ -9619,7 +9619,7 @@
         <v>13.658</v>
       </c>
       <c r="D144" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E144" t="n">
         <v>0.0165361932789285</v>
@@ -9683,7 +9683,7 @@
         <v>13.914</v>
       </c>
       <c r="D145" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E145" t="n">
         <v>0.0186676459464554</v>
@@ -9747,7 +9747,7 @@
         <v>16.308</v>
       </c>
       <c r="D146" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E146" t="n">
         <v>0.0306573950996001</v>
@@ -9811,7 +9811,7 @@
         <v>13.351</v>
       </c>
       <c r="D147" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E147" t="n">
         <v>0.0308126996193702</v>
@@ -9875,7 +9875,7 @@
         <v>9.706</v>
       </c>
       <c r="D148" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E148" t="n">
         <v>0.0218221757095307</v>
@@ -9939,7 +9939,7 @@
         <v>6.963</v>
       </c>
       <c r="D149" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E149" t="n">
         <v>0.0302650726710756</v>
@@ -10003,7 +10003,7 @@
         <v>6.949</v>
       </c>
       <c r="D150" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E150" t="n">
         <v>0.041624091216363</v>
@@ -10067,7 +10067,7 @@
         <v>11.078</v>
       </c>
       <c r="D151" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E151" t="n">
         <v>0.0269036187867944</v>
@@ -10131,7 +10131,7 @@
         <v>10.815</v>
       </c>
       <c r="D152" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E152" t="n">
         <v>0.0509024809580296</v>
@@ -10195,7 +10195,7 @@
         <v>8.762</v>
       </c>
       <c r="D153" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E153" t="n">
         <v>0.060303061036393</v>
@@ -10259,7 +10259,7 @@
         <v>7.184</v>
       </c>
       <c r="D154" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E154" t="n">
         <v>0.07403325925891591</v>
@@ -10323,7 +10323,7 @@
         <v>6.614</v>
       </c>
       <c r="D155" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E155" t="n">
         <v>0.0616220988643666</v>
@@ -10387,7 +10387,7 @@
         <v>6.402</v>
       </c>
       <c r="D156" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E156" t="n">
         <v>0.0516710562321046</v>
@@ -10451,7 +10451,7 @@
         <v>6.684</v>
       </c>
       <c r="D157" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E157" t="n">
         <v>0.028721463944142</v>
@@ -10515,7 +10515,7 @@
         <v>6.674</v>
       </c>
       <c r="D158" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E158" t="n">
         <v>0.0321057226198415</v>
@@ -10579,7 +10579,7 @@
         <v>6.191</v>
       </c>
       <c r="D159" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E159" t="n">
         <v>0.023278960880513</v>
@@ -10643,7 +10643,7 @@
         <v>7.564</v>
       </c>
       <c r="D160" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E160" t="n">
         <v>0.021518613367031</v>
@@ -10707,7 +10707,7 @@
         <v>7.131</v>
       </c>
       <c r="D161" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E161" t="n">
         <v>0.0206897942504535</v>
@@ -10771,7 +10771,7 @@
         <v>6.094</v>
       </c>
       <c r="D162" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E162" t="n">
         <v>0.0165280015983929</v>
@@ -10835,7 +10835,7 @@
         <v>7.555</v>
       </c>
       <c r="D163" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E163" t="n">
         <v>0.0144678792955043</v>
@@ -10899,7 +10899,7 @@
         <v>8.025</v>
       </c>
       <c r="D164" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E164" t="n">
         <v>0.0247589193750172</v>
@@ -10963,7 +10963,7 @@
         <v>9.25</v>
       </c>
       <c r="D165" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E165" t="n">
         <v>0.0169958399686341</v>
@@ -11027,7 +11027,7 @@
         <v>9.704000000000001</v>
       </c>
       <c r="D166" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E166" t="n">
         <v>0.1522324680505942</v>
@@ -11091,7 +11091,7 @@
         <v>9.952999999999999</v>
       </c>
       <c r="D167" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E167" t="n">
         <v>0.0451544088621934</v>
@@ -11155,7 +11155,7 @@
         <v>13.463</v>
       </c>
       <c r="D168" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E168" t="n">
         <v>0.0349900272364417</v>
@@ -11219,7 +11219,7 @@
         <v>17.393</v>
       </c>
       <c r="D169" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E169" t="n">
         <v>0.0683920344648262</v>
@@ -11283,7 +11283,7 @@
         <v>16.596</v>
       </c>
       <c r="D170" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E170" t="n">
         <v>0.0364305294351652</v>
@@ -11347,7 +11347,7 @@
         <v>16.134</v>
       </c>
       <c r="D171" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E171" t="n">
         <v>0.0233116964033494</v>
@@ -11411,7 +11411,7 @@
         <v>17.579</v>
       </c>
       <c r="D172" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E172" t="n">
         <v>0.0246644880001743</v>
@@ -11475,7 +11475,7 @@
         <v>19.251</v>
       </c>
       <c r="D173" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E173" t="n">
         <v>0.0258918775555988</v>
@@ -11539,7 +11539,7 @@
         <v>19.474</v>
       </c>
       <c r="D174" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E174" t="n">
         <v>0.0300874154393871</v>
@@ -11603,7 +11603,7 @@
         <v>19.159</v>
       </c>
       <c r="D175" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E175" t="n">
         <v>0.0242456276124964</v>
@@ -11667,7 +11667,7 @@
         <v>20.366</v>
       </c>
       <c r="D176" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E176" t="n">
         <v>0.0290972011862322</v>
@@ -11731,7 +11731,7 @@
         <v>45.42</v>
       </c>
       <c r="D177" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E177" t="n">
         <v>0.09652126580476759</v>
@@ -11795,7 +11795,7 @@
         <v>42.508</v>
       </c>
       <c r="D178" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E178" t="n">
         <v>0.0804055018040041</v>
@@ -11859,7 +11859,7 @@
         <v>39.196</v>
       </c>
       <c r="D179" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E179" t="n">
         <v>0.038164016790688</v>
@@ -11923,7 +11923,7 @@
         <v>40.246</v>
       </c>
       <c r="D180" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E180" t="n">
         <v>0.0184326822248597</v>
@@ -11987,7 +11987,7 @@
         <v>39.995</v>
       </c>
       <c r="D181" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E181" t="n">
         <v>0.0214769813464954</v>
@@ -12051,7 +12051,7 @@
         <v>36.857</v>
       </c>
       <c r="D182" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E182" t="n">
         <v>0.0387313186656683</v>
@@ -12115,7 +12115,7 @@
         <v>36.952</v>
       </c>
       <c r="D183" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E183" t="n">
         <v>0.0329435614403337</v>
@@ -12179,7 +12179,7 @@
         <v>33.435</v>
       </c>
       <c r="D184" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E184" t="n">
         <v>0.0142138538261254</v>
@@ -12243,7 +12243,7 @@
         <v>33.624</v>
       </c>
       <c r="D185" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E185" t="n">
         <v>0.0251793028243506</v>
@@ -12307,7 +12307,7 @@
         <v>44.492</v>
       </c>
       <c r="D186" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E186" t="n">
         <v>0.0280384281650185</v>
@@ -12371,7 +12371,7 @@
         <v>42.892</v>
       </c>
       <c r="D187" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E187" t="n">
         <v>0.0604256342630834</v>
@@ -12435,7 +12435,7 @@
         <v>37.279</v>
       </c>
       <c r="D188" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E188" t="n">
         <v>0.0808185413479805</v>
@@ -12499,7 +12499,7 @@
         <v>35.638</v>
       </c>
       <c r="D189" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E189" t="n">
         <v>0.1094635815049211</v>
@@ -12563,7 +12563,7 @@
         <v>33.415</v>
       </c>
       <c r="D190" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E190" t="n">
         <v>0.08547515422105791</v>
@@ -12627,7 +12627,7 @@
         <v>33.733</v>
       </c>
       <c r="D191" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E191" t="n">
         <v>0.0631817947141826</v>
@@ -12691,7 +12691,7 @@
         <v>32.367</v>
       </c>
       <c r="D192" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E192" t="n">
         <v>0.0343888537803043</v>
@@ -12755,7 +12755,7 @@
         <v>36.034</v>
       </c>
       <c r="D193" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E193" t="n">
         <v>0.0203754350853462</v>
@@ -12819,7 +12819,7 @@
         <v>31.6</v>
       </c>
       <c r="D194" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E194" t="n">
         <v>0.0267734453082084</v>
@@ -12883,7 +12883,7 @@
         <v>33.903</v>
       </c>
       <c r="D195" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E195" t="n">
         <v>0.019045710330829</v>
@@ -12947,7 +12947,7 @@
         <v>32.574</v>
       </c>
       <c r="D196" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E196" t="n">
         <v>0.0212852933909744</v>
@@ -13011,7 +13011,7 @@
         <v>26.296</v>
       </c>
       <c r="D197" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E197" t="n">
         <v>0.0173874391863743</v>
@@ -13075,7 +13075,7 @@
         <v>28.662</v>
       </c>
       <c r="D198" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E198" t="n">
         <v>0.0204131393887412</v>
@@ -13139,7 +13139,7 @@
         <v>28.454</v>
       </c>
       <c r="D199" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E199" t="n">
         <v>0.0290730854418749</v>
@@ -13203,7 +13203,7 @@
         <v>26.412</v>
       </c>
       <c r="D200" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E200" t="n">
         <v>0.0367292952723801</v>
@@ -13267,7 +13267,7 @@
         <v>25.612</v>
       </c>
       <c r="D201" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E201" t="n">
         <v>0.0389065359874318</v>
@@ -13331,7 +13331,7 @@
         <v>25.413</v>
       </c>
       <c r="D202" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E202" t="n">
         <v>0.0372228318980584</v>
@@ -13395,7 +13395,7 @@
         <v>24.21</v>
       </c>
       <c r="D203" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E203" t="n">
         <v>0.062980786897242</v>
@@ -13459,7 +13459,7 @@
         <v>24.555</v>
       </c>
       <c r="D204" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E204" t="n">
         <v>0.0989968525245785</v>
@@ -13523,7 +13523,7 @@
         <v>23.371</v>
       </c>
       <c r="D205" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E205" t="n">
         <v>0.0376163247274234</v>
@@ -13587,7 +13587,7 @@
         <v>20.787</v>
       </c>
       <c r="D206" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E206" t="n">
         <v>0.0388001215178519</v>
@@ -13651,7 +13651,7 @@
         <v>21.229</v>
       </c>
       <c r="D207" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E207" t="n">
         <v>0.0379206480768819</v>
@@ -13715,7 +13715,7 @@
         <v>22.135</v>
       </c>
       <c r="D208" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E208" t="n">
         <v>0.0260776863045369</v>
@@ -13779,7 +13779,7 @@
         <v>22.16</v>
       </c>
       <c r="D209" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E209" t="n">
         <v>0.0305896863186111</v>
@@ -13843,7 +13843,7 @@
         <v>21.426</v>
       </c>
       <c r="D210" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E210" t="n">
         <v>0.0588593821351727</v>
@@ -13907,7 +13907,7 @@
         <v>20.472</v>
       </c>
       <c r="D211" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E211" t="n">
         <v>0.0486756829389681</v>
@@ -13971,7 +13971,7 @@
         <v>0.544</v>
       </c>
       <c r="D212" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E212" t="n">
         <v>121.2444051106771</v>
@@ -14035,7 +14035,7 @@
         <v>1.476</v>
       </c>
       <c r="D213" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E213" t="n">
         <v>149.4545478820802</v>
@@ -14099,7 +14099,7 @@
         <v>1.397</v>
       </c>
       <c r="D214" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E214" t="n">
         <v>84.01630846659343</v>
@@ -14163,7 +14163,7 @@
         <v>1.292</v>
       </c>
       <c r="D215" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E215" t="n">
         <v>101.6827818552653</v>
@@ -14227,7 +14227,7 @@
         <v>1.185</v>
       </c>
       <c r="D216" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E216" t="n">
         <v>99.04823048909503</v>
@@ -14291,7 +14291,7 @@
         <v>1.111</v>
       </c>
       <c r="D217" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E217" t="n">
         <v>85.5373369852702</v>
@@ -14355,7 +14355,7 @@
         <v>1.025</v>
       </c>
       <c r="D218" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E218" t="n">
         <v>74.67454210917155</v>
@@ -14419,7 +14419,7 @@
         <v>0.917</v>
       </c>
       <c r="D219" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E219" t="n">
         <v>50.9146931966146</v>
@@ -14483,7 +14483,7 @@
         <v>0.863</v>
       </c>
       <c r="D220" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E220" t="n">
         <v>68.46944268544515</v>
@@ -14547,7 +14547,7 @@
         <v>0.83</v>
       </c>
       <c r="D221" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E221" t="n">
         <v>73.97799110412599</v>
@@ -14611,7 +14611,7 @@
         <v>1.547</v>
       </c>
       <c r="D222" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E222" t="n">
         <v>57.41528511047364</v>
@@ -14675,7 +14675,7 @@
         <v>2.087</v>
       </c>
       <c r="D223" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E223" t="n">
         <v>168.8291734059652</v>
@@ -14739,7 +14739,7 @@
         <v>2.222</v>
       </c>
       <c r="D224" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E224" t="n">
         <v>156.0421670277914</v>
@@ -14803,7 +14803,7 @@
         <v>2.803</v>
       </c>
       <c r="D225" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E225" t="n">
         <v>176.3015632629394</v>
@@ -14867,7 +14867,7 @@
         <v>2.607</v>
       </c>
       <c r="D226" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E226" t="n">
         <v>129.3962364196776</v>
@@ -14931,7 +14931,7 @@
         <v>2.512</v>
       </c>
       <c r="D227" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E227" t="n">
         <v>101.5389893849691</v>
@@ -14995,7 +14995,7 @@
         <v>2.406</v>
       </c>
       <c r="D228" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E228" t="n">
         <v>104.0353469848633</v>
@@ -15059,7 +15059,7 @@
         <v>2.407</v>
       </c>
       <c r="D229" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E229" t="n">
         <v>93.73795509338376</v>
@@ -15123,7 +15123,7 @@
         <v>2.496</v>
       </c>
       <c r="D230" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E230" t="n">
         <v>81.19649124145508</v>
@@ -15187,7 +15187,7 @@
         <v>2.512</v>
       </c>
       <c r="D231" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E231" t="n">
         <v>83.10185750325522</v>
@@ -15251,7 +15251,7 @@
         <v>2.601</v>
       </c>
       <c r="D232" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E232" t="n">
         <v>84.17017555236818</v>
@@ -15315,7 +15315,7 @@
         <v>2.609</v>
       </c>
       <c r="D233" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E233" t="n">
         <v>90.0953877766927</v>
@@ -15379,7 +15379,7 @@
         <v>2.706</v>
       </c>
       <c r="D234" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E234" t="n">
         <v>81.47523371378583</v>
@@ -15443,7 +15443,7 @@
         <v>3.523</v>
       </c>
       <c r="D235" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E235" t="n">
         <v>83.03660519917806</v>
@@ -15507,7 +15507,7 @@
         <v>2.799</v>
       </c>
       <c r="D236" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E236" t="n">
         <v>100.2915852864583</v>
@@ -15571,7 +15571,7 @@
         <v>2.904</v>
       </c>
       <c r="D237" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E237" t="n">
         <v>105.9536450703939</v>
@@ -15635,7 +15635,7 @@
         <v>2.908</v>
       </c>
       <c r="D238" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E238" t="n">
         <v>98.67868804931636</v>
@@ -15699,7 +15699,7 @@
         <v>2.888</v>
       </c>
       <c r="D239" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E239" t="n">
         <v>107.377311706543</v>
@@ -15763,7 +15763,7 @@
         <v>2.813</v>
       </c>
       <c r="D240" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E240" t="n">
         <v>98.5529073079427</v>
@@ -15827,7 +15827,7 @@
         <v>2.789</v>
       </c>
       <c r="D241" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E241" t="n">
         <v>90.94625282287596</v>
@@ -15891,7 +15891,7 @@
         <v>2.808</v>
       </c>
       <c r="D242" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E242" t="n">
         <v>77.29380416870116</v>
@@ -15955,7 +15955,7 @@
         <v>2.904</v>
       </c>
       <c r="D243" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E243" t="n">
         <v>82.07023620605467</v>
@@ -16019,7 +16019,7 @@
         <v>4.093</v>
       </c>
       <c r="D244" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E244" t="n">
         <v>157.5831934611003</v>
@@ -16083,7 +16083,7 @@
         <v>4.536</v>
       </c>
       <c r="D245" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E245" t="n">
         <v>121.7112553914388</v>
@@ -16147,7 +16147,7 @@
         <v>4.932</v>
       </c>
       <c r="D246" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E246" t="n">
         <v>134.4527511596681</v>
@@ -16211,7 +16211,7 @@
         <v>11.165</v>
       </c>
       <c r="D247" t="n">
-        <v>53.60263331259628</v>
+        <v>74.13045382239731</v>
       </c>
       <c r="E247" t="n">
         <v>0.0387812045713265</v>
@@ -16275,7 +16275,7 @@
         <v>9.048</v>
       </c>
       <c r="D248" t="n">
-        <v>74.36527332853694</v>
+        <v>61.37992573078208</v>
       </c>
       <c r="E248" t="n">
         <v>0.0531226196326315</v>
@@ -16339,7 +16339,7 @@
         <v>7.329</v>
       </c>
       <c r="D249" t="n">
-        <v>87.57179823606837</v>
+        <v>67.53912162715449</v>
       </c>
       <c r="E249" t="n">
         <v>0.0486216112816085</v>
@@ -16403,7 +16403,7 @@
         <v>5.75</v>
       </c>
       <c r="D250" t="n">
-        <v>90.81639773325251</v>
+        <v>51.23371358902412</v>
       </c>
       <c r="E250" t="n">
         <v>0.0339860008874287</v>
@@ -16467,7 +16467,7 @@
         <v>6.265</v>
       </c>
       <c r="D251" t="n">
-        <v>71.4530669145032</v>
+        <v>43.35518271124661</v>
       </c>
       <c r="E251" t="n">
         <v>0.0307271035853773</v>
@@ -16531,7 +16531,7 @@
         <v>8.446999999999999</v>
       </c>
       <c r="D252" t="n">
-        <v>73.41070654004763</v>
+        <v>60.52961754946105</v>
       </c>
       <c r="E252" t="n">
         <v>0.0248378882727896</v>
@@ -16595,7 +16595,7 @@
         <v>8.532</v>
       </c>
       <c r="D253" t="n">
-        <v>60.06634450960263</v>
+        <v>46.11203016608268</v>
       </c>
       <c r="E253" t="n">
         <v>0.0304903762880712</v>
@@ -16659,7 +16659,7 @@
         <v>7.938</v>
       </c>
       <c r="D254" t="n">
-        <v>76.88629496202944</v>
+        <v>53.90419197731964</v>
       </c>
       <c r="E254" t="n">
         <v>0.0316075270529836</v>
@@ -16723,7 +16723,7 @@
         <v>6.029</v>
       </c>
       <c r="D255" t="n">
-        <v>56.67038553908898</v>
+        <v>36.67356938706484</v>
       </c>
       <c r="E255" t="n">
         <v>0.0326576187896231</v>
@@ -16787,7 +16787,7 @@
         <v>4.275</v>
       </c>
       <c r="D256" t="n">
-        <v>79.07465979997086</v>
+        <v>35.27100032176562</v>
       </c>
       <c r="E256" t="n">
         <v>0.0237237591839706</v>
@@ -16851,7 +16851,7 @@
         <v>6.721</v>
       </c>
       <c r="D257" t="n">
-        <v>97.81879097378548</v>
+        <v>59.16717006798063</v>
       </c>
       <c r="E257" t="n">
         <v>0.0201966421833882</v>
@@ -16915,7 +16915,7 @@
         <v>6.723</v>
       </c>
       <c r="D258" t="n">
-        <v>126.0428302904788</v>
+        <v>94.04825693640974</v>
       </c>
       <c r="E258" t="n">
         <v>0.0358721808297559</v>
@@ -16979,7 +16979,7 @@
         <v>7.488</v>
       </c>
       <c r="D259" t="n">
-        <v>89.81203567263958</v>
+        <v>64.79832520039118</v>
       </c>
       <c r="E259" t="n">
         <v>0.0487280866752068</v>
@@ -17043,7 +17043,7 @@
         <v>7.28</v>
       </c>
       <c r="D260" t="n">
-        <v>86.30412226814997</v>
+        <v>59.63733275547654</v>
       </c>
       <c r="E260" t="n">
         <v>0.0767023862960437</v>
@@ -17107,7 +17107,7 @@
         <v>6.235</v>
       </c>
       <c r="D261" t="n">
-        <v>80.32233111229525</v>
+        <v>56.28180320594232</v>
       </c>
       <c r="E261" t="n">
         <v>0.0528563571472963</v>
@@ -17171,7 +17171,7 @@
         <v>5.773</v>
       </c>
       <c r="D262" t="n">
-        <v>85.99467467015457</v>
+        <v>69.7245750583298</v>
       </c>
       <c r="E262" t="n">
         <v>0.055581181930999</v>
@@ -17235,7 +17235,7 @@
         <v>7.296</v>
       </c>
       <c r="D263" t="n">
-        <v>85.09813030069525</v>
+        <v>74.98381957837482</v>
       </c>
       <c r="E263" t="n">
         <v>0.0432414657746752</v>
@@ -17299,7 +17299,7 @@
         <v>7.311</v>
       </c>
       <c r="D264" t="n">
-        <v>109.9001670836911</v>
+        <v>153.1303579649171</v>
       </c>
       <c r="E264" t="n">
         <v>0.04439690321063</v>
@@ -17363,7 +17363,7 @@
         <v>6.278</v>
       </c>
       <c r="D265" t="n">
-        <v>121.312223132744</v>
+        <v>152.6608768924711</v>
       </c>
       <c r="E265" t="n">
         <v>0.0567478865074615</v>
@@ -17427,7 +17427,7 @@
         <v>6.347</v>
       </c>
       <c r="D266" t="n">
-        <v>125.9892774091345</v>
+        <v>191.1911396095693</v>
       </c>
       <c r="E266" t="n">
         <v>0.0446980871492997</v>
@@ -17491,7 +17491,7 @@
         <v>5.566</v>
       </c>
       <c r="D267" t="n">
-        <v>139.7148151603081</v>
+        <v>161.8097544913446</v>
       </c>
       <c r="E267" t="n">
         <v>0.0623312025951842</v>
@@ -17555,7 +17555,7 @@
         <v>7.828</v>
       </c>
       <c r="D268" t="n">
-        <v>106.6895134623232</v>
+        <v>153.45054409492</v>
       </c>
       <c r="E268" t="n">
         <v>0.0296544635978837</v>
@@ -17619,7 +17619,7 @@
         <v>8.079000000000001</v>
       </c>
       <c r="D269" t="n">
-        <v>83.86807369886057</v>
+        <v>117.6281682872267</v>
       </c>
       <c r="E269" t="n">
         <v>0.0491366248267392</v>
@@ -17683,7 +17683,7 @@
         <v>7.501</v>
       </c>
       <c r="D270" t="n">
-        <v>79.56630150635979</v>
+        <v>120.9294572194867</v>
       </c>
       <c r="E270" t="n">
         <v>0.0225378795682142</v>
@@ -17747,7 +17747,7 @@
         <v>8.178000000000001</v>
       </c>
       <c r="D271" t="n">
-        <v>87.2331363980304</v>
+        <v>120.6786023914649</v>
       </c>
       <c r="E271" t="n">
         <v>0.0440807589329779</v>
@@ -17811,7 +17811,7 @@
         <v>7.766</v>
       </c>
       <c r="D272" t="n">
-        <v>89.94130010547372</v>
+        <v>130.2887371307345</v>
       </c>
       <c r="E272" t="n">
         <v>0.0266834201368813</v>
@@ -17875,7 +17875,7 @@
         <v>8.936999999999999</v>
       </c>
       <c r="D273" t="n">
-        <v>108.7925514509114</v>
+        <v>187.0305839557435</v>
       </c>
       <c r="E273" t="n">
         <v>0.0232152248499915</v>
@@ -17939,7 +17939,7 @@
         <v>11.107</v>
       </c>
       <c r="D274" t="n">
-        <v>187.461532478308</v>
+        <v>271.5174513551767</v>
       </c>
       <c r="E274" t="n">
         <v>0.0238104355133449</v>
@@ -18003,7 +18003,7 @@
         <v>14.356</v>
       </c>
       <c r="D275" t="n">
-        <v>143.8253350767924</v>
+        <v>197.6547345290266</v>
       </c>
       <c r="E275" t="n">
         <v>0.0296325676220779</v>
@@ -18067,7 +18067,7 @@
         <v>14.862</v>
       </c>
       <c r="D276" t="n">
-        <v>240.3952968731671</v>
+        <v>299.2009229902017</v>
       </c>
       <c r="E276" t="n">
         <v>0.0343204368061075</v>
@@ -18131,7 +18131,7 @@
         <v>14.211</v>
       </c>
       <c r="D277" t="n">
-        <v>240.3952968731671</v>
+        <v>301.1719445906172</v>
       </c>
       <c r="E277" t="n">
         <v>0.0260544235352426</v>
@@ -18195,7 +18195,7 @@
         <v>15.009</v>
       </c>
       <c r="D278" t="n">
-        <v>240.3952968731671</v>
+        <v>423.4053185372721</v>
       </c>
       <c r="E278" t="n">
         <v>0.0454797817704578</v>
@@ -18259,7 +18259,7 @@
         <v>15.79</v>
       </c>
       <c r="D279" t="n">
-        <v>240.3952968731671</v>
+        <v>409.5913303820856</v>
       </c>
       <c r="E279" t="n">
         <v>0.0290344501845538</v>
@@ -18323,7 +18323,7 @@
         <v>15.624</v>
       </c>
       <c r="D280" t="n">
-        <v>240.3952968731671</v>
+        <v>378.5688834266829</v>
       </c>
       <c r="E280" t="n">
         <v>0.047092413646169</v>
@@ -18387,7 +18387,7 @@
         <v>14.841</v>
       </c>
       <c r="D281" t="n">
-        <v>240.3952968731671</v>
+        <v>367.5545195023332</v>
       </c>
       <c r="E281" t="n">
         <v>0.0306681161746382</v>

</xml_diff>